<commit_message>
Corte MPOO: correccion aceptada de una P00 y P02 (ya compila y los .class son reales)
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P02-corte-07sep.xlsx
+++ b/calificaciones/P00-P02-corte-07sep.xlsx
@@ -8,14 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Matriz" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="323297291" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="322098930" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="323290577" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="322179684" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="322330157" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="322153686" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="426058988" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="323272733" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="322098930" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="323290577" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="322179684" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="322330157" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="322153686" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="426058988" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="323272733" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -125,12 +124,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
+        <fgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -177,10 +176,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -655,9 +654,9 @@
           <t>323297291</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -665,14 +664,14 @@
           <t>10</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>P00 vacia y P02 no compila. Ver tu hoja.</t>
+          <t>Corregida y aceptada. Tu P02 ya compila y tus .class son reales. Detalle: te quedo un prueba.txt vacio en p02, borralo.</t>
         </is>
       </c>
     </row>
@@ -709,7 +708,7 @@
           <t>323072461</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
@@ -719,7 +718,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
@@ -773,7 +772,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
@@ -790,17 +789,17 @@
           <t>424020705</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
@@ -881,7 +880,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
@@ -908,7 +907,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
@@ -925,17 +924,17 @@
           <t>321094427</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
@@ -952,17 +951,17 @@
           <t>316087045</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
@@ -989,7 +988,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
@@ -1033,7 +1032,7 @@
           <t>322330157</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
@@ -1060,7 +1059,7 @@
           <t>426058256</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
@@ -1141,17 +1140,17 @@
           <t>319112375</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
@@ -1205,7 +1204,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
@@ -1222,17 +1221,17 @@
           <t>119005277</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
@@ -1276,7 +1275,7 @@
           <t>322153686</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
@@ -1303,17 +1302,17 @@
           <t>321337964</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
@@ -1330,7 +1329,7 @@
           <t>426058988</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
@@ -1357,7 +1356,7 @@
           <t>322095458</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>NP</t>
         </is>
@@ -1384,7 +1383,7 @@
           <t>323272733</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
@@ -1460,7 +1459,7 @@
       </c>
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -1470,7 +1469,7 @@
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1481,7 @@
       </c>
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1492,7 +1491,7 @@
       </c>
       <c r="D40" s="13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1520,7 @@
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>Las tres completas y correctas: 10 de 29     ·     Sin ninguna entrega: 6 de 29</t>
+          <t>Las tres completas y correctas: 11 de 29     ·     Sin ninguna entrega: 6 de 29</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1546,21 +1545,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 323297291</t>
+          <t>Correccion · 322098930</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 323297291   ·   Practicas por corregir: P00 y P02</t>
+          <t>Cuenta: 322098930   ·   Practicas por corregir: P02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: PC      P01: 10      P02: PC</t>
+          <t>P00: 10      P01: 10      P02: PC</t>
         </is>
       </c>
     </row>
@@ -1579,102 +1578,78 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu P00 esta vacio: el archivo pesa 1 byte. Tu nombre esta en el nombre del archivo, pero adentro no hay nada.</t>
+          <t>Uno de tus tres ejemplos es el Circulo del ejemplo que vimos en clase, copiado. Ademas esa clase solo declara atributos: no tiene ni un metodo y nunca usa el radio.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Abre tu archivo de p00, escribe adentro tu nombre completo, guarda y vuelve a hacer push.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="56" customHeight="1">
+          <t>Sustituyelo por un objeto tuyo, distinto al de la demo, con al menos un metodo que use sus atributos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu P02 no compila. Los archivos se llaman ejemploN.java pero las clases de adentro se llaman Punto y PruebaPunto: Java exige que el archivo se llame igual que la clase publica.</t>
+          <t>Tu codigo trae comentarios que te explican el ejercicio a ti (del tipo 'en la imagen de tu guia dice x.x = 2 por error tipografico, cambialo').</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Renombra cada archivo al nombre de su clase (Punto.java, PruebaPunto.java). Deja UNA sola clase Punto y UNA sola PruebaPunto: ahora tienes Punto repetida en dos archivos y PruebaPunto en tres.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>En uno de tus archivos hay un error de escritura: Punto p new = Punto (5, 8);</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Se escribe: Punto p = new Punto(5, 8);</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="56" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Tus 5 archivos .class de la P02 no son archivos compilados: son los .java con la extension cambiada.</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>El .class lo genera la computadora, no se renombra a mano. Corre javac Punto.java PruebaPunto.java y sube los .class que aparezcan. Tu HolaMundo.class de la P01 si es correcto: hazlo igual.</t>
+          <t>Esos comentarios no los escribiste tu. Lo que se califica es que entiendas tu codigo: borralos y escribe con tus palabras que hace cada parte. Tus ejemplos 1 y 2 si estan bien.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>git checkout TU-RAMA</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git commit -m "Correccion PNN"</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
+          <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>git commit -m "Correccion PNN"</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Tu rama y tu carpeta llevan tu apellido y tu nombre. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -1701,14 +1676,14 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 322098930</t>
+          <t>Correccion · 323290577</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 322098930   ·   Practicas por corregir: P02</t>
+          <t>Cuenta: 323290577   ·   Practicas por corregir: P02</t>
         </is>
       </c>
     </row>
@@ -1734,24 +1709,24 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Uno de tus tres ejemplos es el Circulo del ejemplo que vimos en clase, copiado. Ademas esa clase solo declara atributos: no tiene ni un metodo y nunca usa el radio.</t>
+          <t>Tu carpeta no compila. PruebaPunto3 y PruebaPunto4 crean el objeto con new Punto(5,8), pero tu clase Punto no tiene constructor con parametros: ese lo tienen Punto2 y Punto3.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Sustituyelo por un objeto tuyo, distinto al de la demo, con al menos un metodo que use sus atributos.</t>
+          <t>O le agregas a Punto el constructor Punto(int x, int y), o cambias esas pruebas para que usen la clase que si lo tiene.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu codigo trae comentarios que te explican el ejercicio a ti (del tipo 'en la imagen de tu guia dice x.x = 2 por error tipografico, cambialo').</t>
+          <t>Tu PruebaPunto.java arrastra el error de la guia: asigna x.x dos veces y nunca x.y, asi que imprime mal.</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Esos comentarios no los escribiste tu. Lo que se califica es que entiendas tu codigo: borralos y escribe con tus palabras que hace cada parte. Tus ejemplos 1 y 2 si estan bien.</t>
+          <t>La segunda linea debe ser x.y = 2;</t>
         </is>
       </c>
     </row>
@@ -1832,14 +1807,14 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 323290577</t>
+          <t>Correccion · 322179684</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 323290577   ·   Practicas por corregir: P02</t>
+          <t>Cuenta: 322179684   ·   Practicas por corregir: P02</t>
         </is>
       </c>
     </row>
@@ -1862,27 +1837,27 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="56" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu carpeta no compila. PruebaPunto3 y PruebaPunto4 crean el objeto con new Punto(5,8), pero tu clase Punto no tiene constructor con parametros: ese lo tienen Punto2 y Punto3.</t>
+          <t>Tu variante de constructores no compila. Tu clase Punto solo tiene el constructor vacio, y adentro hace this.x = x; this.y = y;, que se asigna a si mismo y no hace nada. Pero tu PruebaPunto llama new Punto(5,8).</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>O le agregas a Punto el constructor Punto(int x, int y), o cambias esas pruebas para que usen la clase que si lo tiene.</t>
+          <t>Agrega el constructor con parametros: Punto(int x, int y) { this.x = x; this.y = y; }  y deja el vacio aparte si lo necesitas.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu PruebaPunto.java arrastra el error de la guia: asigna x.x dos veces y nunca x.y, asi que imprime mal.</t>
+          <t>Tu variante de metodos si compila y esta bien resuelta (incluso corregiste el error de la guia).</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>La segunda linea debe ser x.y = 2;</t>
+          <t>No le muevas: esa quedate como esta.</t>
         </is>
       </c>
     </row>
@@ -1963,21 +1938,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 322179684</t>
+          <t>Correccion · 322330157</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 322179684   ·   Practicas por corregir: P02</t>
+          <t>Cuenta: 322330157   ·   Practicas por corregir: P00 y P01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: 10      P01: 10      P02: PC</t>
+          <t>P00: PC      P01: 9      P02: 10</t>
         </is>
       </c>
     </row>
@@ -1993,27 +1968,27 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="56" customHeight="1">
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu variante de constructores no compila. Tu clase Punto solo tiene el constructor vacio, y adentro hace this.x = x; this.y = y;, que se asigna a si mismo y no hace nada. Pero tu PruebaPunto llama new Punto(5,8).</t>
+          <t>Tu P00 es un HolaMundo.java. La P00 pedia un archivo de texto con tu nombre, que era la prueba de que sabes hacer push.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Agrega el constructor con parametros: Punto(int x, int y) { this.x = x; this.y = y; }  y deja el vacio aparte si lo necesitas.</t>
+          <t>Crea un .txt en tu carpeta de p00 con tu nombre completo adentro, y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu variante de metodos si compila y esta bien resuelta (incluso corregiste el error de la guia).</t>
+          <t>Tu P01 imprime solo 'Hola, mundo': no lleva tu nombre y es practicamente el mismo archivo que dejaste en p00.</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>No le muevas: esa quedate como esta.</t>
+          <t>Modificalo para que imprima tu nombre, como pedia la practica.</t>
         </is>
       </c>
     </row>
@@ -2094,14 +2069,14 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 322330157</t>
+          <t>Correccion · 322153686</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 322330157   ·   Practicas por corregir: P00 y P01</t>
+          <t>Cuenta: 322153686   ·   Practicas por corregir: P00</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2102,7 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu P00 es un HolaMundo.java. La P00 pedia un archivo de texto con tu nombre, que era la prueba de que sabes hacer push.</t>
+          <t>Tu P00 es un HolaMundo.java. La P00 pedia un archivo de texto con tu nombre.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
@@ -2139,12 +2114,12 @@
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu P01 imprime solo 'Hola, mundo': no lleva tu nombre y es practicamente el mismo archivo que dejaste en p00.</t>
+          <t>Tu P01 estaba en una carpeta de un solo digito.</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Modificalo para que imprima tu nombre, como pedia la practica.</t>
+          <t>Ya la normalizamos a dos digitos. No crees otra: trabaja en la que te baja.</t>
         </is>
       </c>
     </row>
@@ -2225,21 +2200,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 322153686</t>
+          <t>Correccion · 426058988</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 322153686   ·   Practicas por corregir: P00</t>
+          <t>Cuenta: 426058988   ·   Practicas por corregir: P00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: PC      P01: 9      P02: 10</t>
+          <t>P00: PC      P01: 10      P02: 10</t>
         </is>
       </c>
     </row>
@@ -2258,24 +2233,24 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu P00 es un HolaMundo.java. La P00 pedia un archivo de texto con tu nombre.</t>
+          <t>Tu P00 no lleva tu nombre: dice 'Practica 00, creo que si es asi unu'. La practica pedia tu nombre para identificar la entrega.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Crea un .txt en tu carpeta de p00 con tu nombre completo adentro, y haz push.</t>
+          <t>Abre ese archivo, escribe tu nombre completo, guarda y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu P01 estaba en una carpeta de un solo digito.</t>
+          <t>Lo guardaste en UTF-16 (le pasa al Bloc de notas de Windows).</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Ya la normalizamos a dos digitos. No crees otra: trabaja en la que te baja.</t>
+          <t>Al guardar, elige la codificacion UTF-8. Se lee bien igual, pero es buena costumbre.</t>
         </is>
       </c>
     </row>
@@ -2341,137 +2316,6 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="76" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Correccion · 426058988</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 426058988   ·   Practicas por corregir: P00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: PC      P01: 10      P02: 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>Tu P00 no lleva tu nombre: dice 'Practica 00, creo que si es asi unu'. La practica pedia tu nombre para identificar la entrega.</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Abre ese archivo, escribe tu nombre completo, guarda y haz push.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Lo guardaste en UTF-16 (le pasa al Bloc de notas de Windows).</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>Al guardar, elige la codificacion UTF-8. Se lee bien igual, pero es buena costumbre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>git commit -m "Correccion PNN"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>Tu rama y tu carpeta llevan tu apellido y tu nombre. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Corte MPOO: una P02 corregida y aceptada
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P02-corte-07sep.xlsx
+++ b/calificaciones/P00-P02-corte-07sep.xlsx
@@ -8,13 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Matriz" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="322098930" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="323290577" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="322179684" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="322330157" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="322153686" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="426058988" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="323272733" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="323290577" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="322179684" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="322330157" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="322153686" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="426058988" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="323272733" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -772,14 +771,14 @@
           <t>10</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>En la P02, uno de los ejemplos es el de la demo de clase copiado. Ver tu hoja.</t>
+          <t>Corregida y aceptada. Sustituiste el ejemplo de la demo por uno propio y quitaste los comentarios que no eran tuyos. Los tres ejemplos compilan.</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1468,7 @@
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1490,7 @@
       </c>
       <c r="D40" s="13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1519,7 @@
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>Las tres completas y correctas: 11 de 29     ·     Sin ninguna entrega: 6 de 29</t>
+          <t>Las tres completas y correctas: 12 de 29     ·     Sin ninguna entrega: 6 de 29</t>
         </is>
       </c>
     </row>
@@ -1545,14 +1544,14 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 322098930</t>
+          <t>Correccion · 323290577</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 322098930   ·   Practicas por corregir: P02</t>
+          <t>Cuenta: 323290577   ·   Practicas por corregir: P02</t>
         </is>
       </c>
     </row>
@@ -1578,24 +1577,24 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Uno de tus tres ejemplos es el Circulo del ejemplo que vimos en clase, copiado. Ademas esa clase solo declara atributos: no tiene ni un metodo y nunca usa el radio.</t>
+          <t>Tu carpeta no compila. PruebaPunto3 y PruebaPunto4 crean el objeto con new Punto(5,8), pero tu clase Punto no tiene constructor con parametros: ese lo tienen Punto2 y Punto3.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Sustituyelo por un objeto tuyo, distinto al de la demo, con al menos un metodo que use sus atributos.</t>
+          <t>O le agregas a Punto el constructor Punto(int x, int y), o cambias esas pruebas para que usen la clase que si lo tiene.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu codigo trae comentarios que te explican el ejercicio a ti (del tipo 'en la imagen de tu guia dice x.x = 2 por error tipografico, cambialo').</t>
+          <t>Tu PruebaPunto.java arrastra el error de la guia: asigna x.x dos veces y nunca x.y, asi que imprime mal.</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Esos comentarios no los escribiste tu. Lo que se califica es que entiendas tu codigo: borralos y escribe con tus palabras que hace cada parte. Tus ejemplos 1 y 2 si estan bien.</t>
+          <t>La segunda linea debe ser x.y = 2;</t>
         </is>
       </c>
     </row>
@@ -1676,14 +1675,14 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 323290577</t>
+          <t>Correccion · 322179684</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 323290577   ·   Practicas por corregir: P02</t>
+          <t>Cuenta: 322179684   ·   Practicas por corregir: P02</t>
         </is>
       </c>
     </row>
@@ -1706,27 +1705,27 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="56" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu carpeta no compila. PruebaPunto3 y PruebaPunto4 crean el objeto con new Punto(5,8), pero tu clase Punto no tiene constructor con parametros: ese lo tienen Punto2 y Punto3.</t>
+          <t>Tu variante de constructores no compila. Tu clase Punto solo tiene el constructor vacio, y adentro hace this.x = x; this.y = y;, que se asigna a si mismo y no hace nada. Pero tu PruebaPunto llama new Punto(5,8).</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>O le agregas a Punto el constructor Punto(int x, int y), o cambias esas pruebas para que usen la clase que si lo tiene.</t>
+          <t>Agrega el constructor con parametros: Punto(int x, int y) { this.x = x; this.y = y; }  y deja el vacio aparte si lo necesitas.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu PruebaPunto.java arrastra el error de la guia: asigna x.x dos veces y nunca x.y, asi que imprime mal.</t>
+          <t>Tu variante de metodos si compila y esta bien resuelta (incluso corregiste el error de la guia).</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>La segunda linea debe ser x.y = 2;</t>
+          <t>No le muevas: esa quedate como esta.</t>
         </is>
       </c>
     </row>
@@ -1807,21 +1806,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 322179684</t>
+          <t>Correccion · 322330157</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 322179684   ·   Practicas por corregir: P02</t>
+          <t>Cuenta: 322330157   ·   Practicas por corregir: P00 y P01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: 10      P01: 10      P02: PC</t>
+          <t>P00: PC      P01: 9      P02: 10</t>
         </is>
       </c>
     </row>
@@ -1837,27 +1836,27 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="56" customHeight="1">
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu variante de constructores no compila. Tu clase Punto solo tiene el constructor vacio, y adentro hace this.x = x; this.y = y;, que se asigna a si mismo y no hace nada. Pero tu PruebaPunto llama new Punto(5,8).</t>
+          <t>Tu P00 es un HolaMundo.java. La P00 pedia un archivo de texto con tu nombre, que era la prueba de que sabes hacer push.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Agrega el constructor con parametros: Punto(int x, int y) { this.x = x; this.y = y; }  y deja el vacio aparte si lo necesitas.</t>
+          <t>Crea un .txt en tu carpeta de p00 con tu nombre completo adentro, y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu variante de metodos si compila y esta bien resuelta (incluso corregiste el error de la guia).</t>
+          <t>Tu P01 imprime solo 'Hola, mundo': no lleva tu nombre y es practicamente el mismo archivo que dejaste en p00.</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>No le muevas: esa quedate como esta.</t>
+          <t>Modificalo para que imprima tu nombre, como pedia la practica.</t>
         </is>
       </c>
     </row>
@@ -1938,14 +1937,14 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 322330157</t>
+          <t>Correccion · 322153686</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 322330157   ·   Practicas por corregir: P00 y P01</t>
+          <t>Cuenta: 322153686   ·   Practicas por corregir: P00</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1970,7 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu P00 es un HolaMundo.java. La P00 pedia un archivo de texto con tu nombre, que era la prueba de que sabes hacer push.</t>
+          <t>Tu P00 es un HolaMundo.java. La P00 pedia un archivo de texto con tu nombre.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
@@ -1983,12 +1982,12 @@
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu P01 imprime solo 'Hola, mundo': no lleva tu nombre y es practicamente el mismo archivo que dejaste en p00.</t>
+          <t>Tu P01 estaba en una carpeta de un solo digito.</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Modificalo para que imprima tu nombre, como pedia la practica.</t>
+          <t>Ya la normalizamos a dos digitos. No crees otra: trabaja en la que te baja.</t>
         </is>
       </c>
     </row>
@@ -2069,21 +2068,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 322153686</t>
+          <t>Correccion · 426058988</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 322153686   ·   Practicas por corregir: P00</t>
+          <t>Cuenta: 426058988   ·   Practicas por corregir: P00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: PC      P01: 9      P02: 10</t>
+          <t>P00: PC      P01: 10      P02: 10</t>
         </is>
       </c>
     </row>
@@ -2102,24 +2101,24 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu P00 es un HolaMundo.java. La P00 pedia un archivo de texto con tu nombre.</t>
+          <t>Tu P00 no lleva tu nombre: dice 'Practica 00, creo que si es asi unu'. La practica pedia tu nombre para identificar la entrega.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Crea un .txt en tu carpeta de p00 con tu nombre completo adentro, y haz push.</t>
+          <t>Abre ese archivo, escribe tu nombre completo, guarda y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu P01 estaba en una carpeta de un solo digito.</t>
+          <t>Lo guardaste en UTF-16 (le pasa al Bloc de notas de Windows).</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Ya la normalizamos a dos digitos. No crees otra: trabaja en la que te baja.</t>
+          <t>Al guardar, elige la codificacion UTF-8. Se lee bien igual, pero es buena costumbre.</t>
         </is>
       </c>
     </row>
@@ -2185,137 +2184,6 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="76" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Correccion · 426058988</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 426058988   ·   Practicas por corregir: P00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: PC      P01: 10      P02: 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>Tu P00 no lleva tu nombre: dice 'Practica 00, creo que si es asi unu'. La practica pedia tu nombre para identificar la entrega.</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Abre ese archivo, escribe tu nombre completo, guarda y haz push.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Lo guardaste en UTF-16 (le pasa al Bloc de notas de Windows).</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>Al guardar, elige la codificacion UTF-8. Se lee bien igual, pero es buena costumbre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>git commit -m "Correccion PNN"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>Tu rama y tu carpeta llevan tu apellido y tu nombre. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Corte MPOO: entregas recibidas despues del corte, ya consolidadas
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P02-corte-07sep.xlsx
+++ b/calificaciones/P00-P02-corte-07sep.xlsx
@@ -12,8 +12,9 @@
     <sheet name="322179684" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="322330157" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="322153686" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="426058988" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="323272733" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="321337964" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="426058988" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="323272733" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1306,19 +1307,19 @@
           <t>NP</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Sin entregas registradas.</t>
+          <t>Tu P01 y P02 SI llegaron, estaban en tus ramas viejas y ya las pasamos a tu rama de entregas. Tu P01 no lleva tu nombre. Te falta la P00.</t>
         </is>
       </c>
     </row>
@@ -1441,12 +1442,12 @@
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>23 / 29</t>
+          <t>24 / 29</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>20 / 29</t>
+          <t>21 / 29</t>
         </is>
       </c>
     </row>
@@ -1463,12 +1464,12 @@
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
     </row>
@@ -1507,19 +1508,19 @@
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>Las tres completas y correctas: 12 de 29     ·     Sin ninguna entrega: 6 de 29</t>
+          <t>Las tres completas y correctas: 12 de 29     ·     Sin ninguna entrega: 5 de 29</t>
         </is>
       </c>
     </row>
@@ -2058,6 +2059,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="76" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Correccion · 321337964</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 321337964   ·   Practicas por corregir: P01 y P00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>P00: NP      P01: 9      P02: 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Tu P01 imprime solo 'Hola, mundo': no lleva tu nombre, que era lo que pedia la practica.</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Abre tu HolaMundo.java, haz que imprima tu nombre y vuelve a hacer push. Tu P02 esta bien, esa no le muevas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Te falta la P00, que era la tarea de Git.</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Crea entregas/tu_apellido_nombre/p00/prueba.txt con tu nombre completo adentro y haz push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Tus entregas estaban en las ramas p01-Romero y p02-Romero, no en tu rama del semestre.</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Ya las pasamos a entregas_romero_rodolfo. De aqui en adelante trabaja SOLO en esa rama: haz git fetch origin y luego git checkout entregas_romero_rodolfo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>git commit -m "Correccion PNN"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>Tu rama y tu carpeta llevan tu apellido y tu nombre. No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2183,7 +2327,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Corte MPOO: quita de la version publica una referencia que permitia identificar a un alumno
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P02-corte-07sep.xlsx
+++ b/calificaciones/P00-P02-corte-07sep.xlsx
@@ -1319,7 +1319,7 @@
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Tu P01 y P02 SI llegaron, estaban en tus ramas viejas y ya las pasamos a tu rama de entregas. Tu P01 no lleva tu nombre. Te falta la P00.</t>
+          <t>Tu P01 y P02 SI llegaron: estaban en dos ramas viejas y ya las pasamos a tu rama del semestre. Tu P01 no lleva tu nombre. Te falta la P00.</t>
         </is>
       </c>
     </row>
@@ -2126,12 +2126,12 @@
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>Tus entregas estaban en las ramas p01-Romero y p02-Romero, no en tu rama del semestre.</t>
+          <t>Tus entregas estaban en dos ramas viejas, no en tu rama del semestre: por eso no veias tu carpeta.</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>Ya las pasamos a entregas_romero_rodolfo. De aqui en adelante trabaja SOLO en esa rama: haz git fetch origin y luego git checkout entregas_romero_rodolfo.</t>
+          <t>Ya las pasamos a TU-RAMA de entregas. De aqui en adelante trabaja SOLO en esa: git fetch origin y luego git checkout TU-RAMA.</t>
         </is>
       </c>
     </row>

</xml_diff>